<commit_message>
Excel de historias: incorporados los tiempos de CS-48 y CS-62 y la prioridad N de CS-06 hechos en OneDrive
</commit_message>
<xml_diff>
--- a/documentacion/customer-stories/Customer_Stories_PlanB.xlsx
+++ b/documentacion/customer-stories/Customer_Stories_PlanB.xlsx
@@ -16849,7 +16849,7 @@
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="E9" s="6"/>
       <c r="F9" s="6">
@@ -33396,7 +33396,9 @@
       <c r="E19" s="15">
         <v>40</v>
       </c>
-      <c r="F19" s="15"/>
+      <c r="F19" s="15">
+        <v>20</v>
+      </c>
     </row>
     <row r="20" spans="1:6" ht="43.5">
       <c r="A20" s="16">
@@ -39840,14 +39842,18 @@
       <c r="B25" s="11" t="s">
         <v>436</v>
       </c>
-      <c r="C25" s="5"/>
+      <c r="C25" s="5" t="s">
+        <v>165</v>
+      </c>
       <c r="D25" s="5" t="s">
         <v>307</v>
       </c>
       <c r="E25" s="12">
         <v>30</v>
       </c>
-      <c r="F25" s="12"/>
+      <c r="F25" s="12">
+        <v>4</v>
+      </c>
     </row>
     <row r="26" spans="1:6" ht="33" customHeight="1">
       <c r="A26" s="10">
@@ -39857,14 +39863,18 @@
       <c r="B26" s="11" t="s">
         <v>437</v>
       </c>
-      <c r="C26" s="5"/>
+      <c r="C26" s="5" t="s">
+        <v>165</v>
+      </c>
       <c r="D26" s="5" t="s">
         <v>307</v>
       </c>
       <c r="E26" s="12">
         <v>15</v>
       </c>
-      <c r="F26" s="12"/>
+      <c r="F26" s="12">
+        <v>2</v>
+      </c>
     </row>
     <row r="27" spans="1:6" ht="33" customHeight="1">
       <c r="A27" s="10">

</xml_diff>

<commit_message>
Excel de historias: cambios de OneDrive en CS-45, CS-48, CS-61 y CS-62 y objetivos de CS-64 asignados a José con tiempos estimados
</commit_message>
<xml_diff>
--- a/documentacion/customer-stories/Customer_Stories_PlanB.xlsx
+++ b/documentacion/customer-stories/Customer_Stories_PlanB.xlsx
@@ -18152,7 +18152,7 @@
       </c>
       <c r="D67" s="5"/>
       <c r="E67" s="6">
-        <v>0.5</v>
+        <v>6</v>
       </c>
       <c r="F67" s="6">
         <f ca="1">IF(ISREF(INDIRECT("'"&amp;Historias[[#This Row],[Ref]]&amp;"'!A1")),SUMIFS(INDIRECT("'"&amp;Historias[[#This Row],[Ref]]&amp;"'!F:F"),INDIRECT("'"&amp;Historias[[#This Row],[Ref]]&amp;"'!A:A"),"&gt;0")/60,"")</f>
@@ -32016,14 +32016,20 @@
       <c r="B17" s="11" t="s">
         <v>314</v>
       </c>
-      <c r="C17" s="14"/>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D17" s="14" t="s">
         <v>315</v>
       </c>
       <c r="E17" s="15">
         <v>15</v>
       </c>
-      <c r="F17" s="15"/>
+      <c r="F17" s="15">
+        <v>8</v>
+      </c>
     </row>
     <row r="18" spans="1:6" ht="43.5">
       <c r="A18" s="16">
@@ -32033,14 +32039,22 @@
       <c r="B18" s="11" t="s">
         <v>316</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14" t="s">
-        <v>315</v>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>Flavia</t>
+        </is>
       </c>
       <c r="E18" s="15">
         <v>15</v>
       </c>
-      <c r="F18" s="15"/>
+      <c r="F18" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="19" spans="1:6" ht="43.5">
       <c r="A19" s="16">
@@ -32050,12 +32064,20 @@
       <c r="B19" s="11" t="s">
         <v>317</v>
       </c>
-      <c r="C19" s="14"/>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D19" s="14" t="s">
         <v>315</v>
       </c>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
+      <c r="E19" s="15">
+        <v>10</v>
+      </c>
+      <c r="F19" s="15">
+        <v>6</v>
+      </c>
     </row>
     <row r="20" spans="1:6" ht="28.5">
       <c r="A20" s="16">
@@ -32065,12 +32087,20 @@
       <c r="B20" s="11" t="s">
         <v>318</v>
       </c>
-      <c r="C20" s="14"/>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D20" s="14" t="s">
         <v>315</v>
       </c>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
+      <c r="E20" s="15">
+        <v>8</v>
+      </c>
+      <c r="F20" s="15">
+        <v>8</v>
+      </c>
     </row>
     <row r="21" spans="1:6" ht="28.5">
       <c r="A21" s="16">
@@ -32080,12 +32110,20 @@
       <c r="B21" s="11" t="s">
         <v>319</v>
       </c>
-      <c r="C21" s="14"/>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D21" s="14" t="s">
         <v>315</v>
       </c>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
+      <c r="E21" s="15">
+        <v>10</v>
+      </c>
+      <c r="F21" s="15">
+        <v>15</v>
+      </c>
     </row>
     <row r="22" spans="1:6" ht="57.75">
       <c r="A22" s="16">
@@ -33389,7 +33427,11 @@
       <c r="B19" s="11" t="s">
         <v>345</v>
       </c>
-      <c r="C19" s="14"/>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D19" s="14" t="s">
         <v>292</v>
       </c>
@@ -33408,12 +33450,20 @@
       <c r="B20" s="11" t="s">
         <v>346</v>
       </c>
-      <c r="C20" s="14"/>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D20" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
+      <c r="E20" s="15">
+        <v>20</v>
+      </c>
+      <c r="F20" s="15">
+        <v>15</v>
+      </c>
     </row>
     <row r="21" spans="1:6" ht="28.5">
       <c r="A21" s="16">
@@ -33423,12 +33473,20 @@
       <c r="B21" s="11" t="s">
         <v>347</v>
       </c>
-      <c r="C21" s="14"/>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D21" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
+      <c r="E21" s="15">
+        <v>20</v>
+      </c>
+      <c r="F21" s="15">
+        <v>25</v>
+      </c>
     </row>
     <row r="22" spans="1:6" ht="43.5">
       <c r="A22" s="16">
@@ -33438,12 +33496,20 @@
       <c r="B22" s="11" t="s">
         <v>348</v>
       </c>
-      <c r="C22" s="14"/>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D22" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
+      <c r="E22" s="15">
+        <v>25</v>
+      </c>
+      <c r="F22" s="15">
+        <v>10</v>
+      </c>
     </row>
     <row r="23" spans="1:6" ht="28.5">
       <c r="A23" s="16">
@@ -33453,10 +33519,22 @@
       <c r="B23" s="11" t="s">
         <v>349</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="15"/>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="E23" s="15">
+        <v>20</v>
+      </c>
+      <c r="F23" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="24" spans="1:6" ht="43.5">
       <c r="A24" s="16">
@@ -33466,10 +33544,22 @@
       <c r="B24" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="E24" s="15">
+        <v>10</v>
+      </c>
+      <c r="F24" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="25" spans="1:6" ht="28.5">
       <c r="A25" s="16">
@@ -33479,10 +33569,22 @@
       <c r="B25" s="11" t="s">
         <v>351</v>
       </c>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="E25" s="15">
+        <v>20</v>
+      </c>
+      <c r="F25" s="15">
+        <v>10</v>
+      </c>
     </row>
     <row r="26" spans="1:6" ht="43.5">
       <c r="A26" s="16">
@@ -33492,10 +33594,22 @@
       <c r="B26" s="11" t="s">
         <v>352</v>
       </c>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="E26" s="15">
+        <v>5</v>
+      </c>
+      <c r="F26" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="17" t="s">
@@ -39262,14 +39376,20 @@
       <c r="B28" s="11" t="s">
         <v>420</v>
       </c>
-      <c r="C28" s="14"/>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D28" s="14" t="s">
         <v>244</v>
       </c>
       <c r="E28" s="15">
         <v>30</v>
       </c>
-      <c r="F28" s="15"/>
+      <c r="F28" s="15">
+        <v>12</v>
+      </c>
     </row>
     <row r="29" spans="1:6" ht="33" customHeight="1">
       <c r="A29" s="16">
@@ -39279,14 +39399,20 @@
       <c r="B29" s="11" t="s">
         <v>421</v>
       </c>
-      <c r="C29" s="14"/>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D29" s="14" t="s">
         <v>244</v>
       </c>
       <c r="E29" s="15">
         <v>15</v>
       </c>
-      <c r="F29" s="15"/>
+      <c r="F29" s="15">
+        <v>10</v>
+      </c>
     </row>
     <row r="30" spans="1:6" ht="18" customHeight="1">
       <c r="A30" s="16">
@@ -39296,14 +39422,20 @@
       <c r="B30" s="11" t="s">
         <v>422</v>
       </c>
-      <c r="C30" s="14"/>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D30" s="14" t="s">
         <v>244</v>
       </c>
       <c r="E30" s="15">
         <v>10</v>
       </c>
-      <c r="F30" s="15"/>
+      <c r="F30" s="15">
+        <v>4</v>
+      </c>
     </row>
     <row r="31" spans="1:6" ht="33" customHeight="1">
       <c r="A31" s="16">
@@ -39313,14 +39445,20 @@
       <c r="B31" s="11" t="s">
         <v>423</v>
       </c>
-      <c r="C31" s="14"/>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D31" s="14" t="s">
         <v>244</v>
       </c>
       <c r="E31" s="15">
         <v>20</v>
       </c>
-      <c r="F31" s="15"/>
+      <c r="F31" s="15">
+        <v>2</v>
+      </c>
     </row>
     <row r="32" spans="1:6" ht="18" customHeight="1">
       <c r="A32" s="16">
@@ -39330,14 +39468,20 @@
       <c r="B32" s="11" t="s">
         <v>424</v>
       </c>
-      <c r="C32" s="14"/>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D32" s="14" t="s">
         <v>244</v>
       </c>
       <c r="E32" s="15">
         <v>15</v>
       </c>
-      <c r="F32" s="15"/>
+      <c r="F32" s="15">
+        <v>12</v>
+      </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="17" t="s">
@@ -39772,7 +39916,7 @@
         <v>25</v>
       </c>
       <c r="F21" s="12">
-        <v>22</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="33" customHeight="1">
@@ -39825,7 +39969,11 @@
       <c r="B24" s="11" t="s">
         <v>435</v>
       </c>
-      <c r="C24" s="5"/>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="D24" s="5" t="s">
         <v>307</v>
       </c>
@@ -39884,7 +40032,11 @@
       <c r="B27" s="11" t="s">
         <v>438</v>
       </c>
-      <c r="C27" s="5"/>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="D27" s="5" t="s">
         <v>307</v>
       </c>
@@ -39901,14 +40053,20 @@
       <c r="B28" s="11" t="s">
         <v>424</v>
       </c>
-      <c r="C28" s="5"/>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D28" s="5" t="s">
         <v>307</v>
       </c>
       <c r="E28" s="12">
-        <v>15</v>
-      </c>
-      <c r="F28" s="12"/>
+        <v>5</v>
+      </c>
+      <c r="F28" s="12">
+        <v>2</v>
+      </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="21" t="s">
@@ -40716,8 +40874,14 @@
         <v>455</v>
       </c>
       <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="12"/>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E17" s="12">
+        <v>15</v>
+      </c>
       <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:6" ht="33" customHeight="1">
@@ -40729,8 +40893,14 @@
         <v>456</v>
       </c>
       <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="12"/>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E18" s="12">
+        <v>20</v>
+      </c>
       <c r="F18" s="12"/>
     </row>
     <row r="19" spans="1:6" ht="33" customHeight="1">
@@ -40742,8 +40912,14 @@
         <v>457</v>
       </c>
       <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="12"/>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E19" s="12">
+        <v>25</v>
+      </c>
       <c r="F19" s="12"/>
     </row>
     <row r="20" spans="1:6" ht="18" customHeight="1">
@@ -40755,8 +40931,14 @@
         <v>458</v>
       </c>
       <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="12"/>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E20" s="12">
+        <v>5</v>
+      </c>
       <c r="F20" s="12"/>
     </row>
     <row r="21" spans="1:6" ht="33" customHeight="1">
@@ -40768,8 +40950,14 @@
         <v>459</v>
       </c>
       <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="12"/>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E21" s="12">
+        <v>15</v>
+      </c>
       <c r="F21" s="12"/>
     </row>
     <row r="22" spans="1:6" ht="33" customHeight="1">
@@ -40781,8 +40969,14 @@
         <v>460</v>
       </c>
       <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="12"/>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E22" s="12">
+        <v>15</v>
+      </c>
       <c r="F22" s="12"/>
     </row>
     <row r="23" spans="1:6" ht="33" customHeight="1">
@@ -40794,8 +40988,14 @@
         <v>461</v>
       </c>
       <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="12"/>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E23" s="12">
+        <v>25</v>
+      </c>
       <c r="F23" s="12"/>
     </row>
     <row r="24" spans="1:6" ht="33" customHeight="1">
@@ -40807,8 +41007,14 @@
         <v>462</v>
       </c>
       <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="12"/>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E24" s="12">
+        <v>15</v>
+      </c>
       <c r="F24" s="12"/>
     </row>
     <row r="25" spans="1:6" ht="33" customHeight="1">
@@ -40820,8 +41026,14 @@
         <v>463</v>
       </c>
       <c r="C25" s="5"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="12"/>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E25" s="12">
+        <v>45</v>
+      </c>
       <c r="F25" s="12"/>
     </row>
     <row r="26" spans="1:6" ht="48" customHeight="1">
@@ -40833,8 +41045,14 @@
         <v>464</v>
       </c>
       <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="12"/>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E26" s="12">
+        <v>25</v>
+      </c>
       <c r="F26" s="12"/>
     </row>
     <row r="27" spans="1:6" ht="33" customHeight="1">
@@ -40846,8 +41064,14 @@
         <v>465</v>
       </c>
       <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="12"/>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E27" s="12">
+        <v>20</v>
+      </c>
       <c r="F27" s="12"/>
     </row>
     <row r="28" spans="1:6" ht="33" customHeight="1">
@@ -40859,8 +41083,14 @@
         <v>466</v>
       </c>
       <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="12"/>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E28" s="12">
+        <v>15</v>
+      </c>
       <c r="F28" s="12"/>
     </row>
     <row r="29" spans="1:6" ht="33" customHeight="1">
@@ -40872,8 +41102,14 @@
         <v>467</v>
       </c>
       <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="12"/>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E29" s="12">
+        <v>35</v>
+      </c>
       <c r="F29" s="12"/>
     </row>
     <row r="30" spans="1:6" ht="48" customHeight="1">
@@ -40885,8 +41121,14 @@
         <v>468</v>
       </c>
       <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="12"/>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E30" s="12">
+        <v>35</v>
+      </c>
       <c r="F30" s="12"/>
     </row>
     <row r="31" spans="1:6" ht="18" customHeight="1">
@@ -40898,8 +41140,14 @@
         <v>469</v>
       </c>
       <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="12"/>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="E31" s="12">
+        <v>30</v>
+      </c>
       <c r="F31" s="12"/>
     </row>
     <row r="32" spans="1:6">
@@ -42347,14 +42595,4 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
-  <scriptId id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01GTZEWCAWIM7TFMIJC5EK6T67Q653ALHS:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9jZXUzNjUtbXkuc2hhcmVwb2ludC5jb20vOnU6L2cvcGVyc29uYWwvam9hcXVpbl9kZXZpY2VudGVhYmFkX3VzcF9jZXVfZXMvSVFBV1F6OHlzUWtYU0s5UDM0ZTdzQ3p5QWRTbTYxSVhqT1Q0SWpWUnFrYmtJbTg"/>
-</scriptIds>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{579C8B5B-9FA1-4985-ACF6-918C4CBEE006}"/>
 </file>
</xml_diff>

<commit_message>
Crear páginas rehace también los enlaces «↑ Índice» para repararlos y el enlace de CS-60 muestra ORGANIZACIÓN INTERNA
</commit_message>
<xml_diff>
--- a/documentacion/customer-stories/Customer_Stories_PlanB.xlsx
+++ b/documentacion/customer-stories/Customer_Stories_PlanB.xlsx
@@ -18288,7 +18288,7 @@
     <hyperlink ref="B60" location="'CS-57'!A1" tooltip="Abrir CS-57" display="EDICIÓN DE EXPERIENCIA" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
     <hyperlink ref="B61" location="'CS-58'!A1" tooltip="Abrir CS-58" display="TRANSPORTE PÚBLICO DE LA EXPERIENCIA" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
     <hyperlink ref="B62" location="'CS-59'!A1" tooltip="Abrir CS-59" display="CREAR UNA CUENTA" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="B63" location="'CS-60'!A1" tooltip="Abrir CS-60" display="METODOLOGÍA" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="B63" location="'CS-60'!A1" tooltip="Abrir CS-60" display="ORGANIZACIÓN INTERNA" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
     <hyperlink ref="B64" location="'CS-61'!A1" tooltip="Abrir CS-61" display="AMISTADES Y SEGUIDORES" xr:uid="{8E909EDD-8C49-4731-949C-37B4000BA286}"/>
     <hyperlink ref="B65" location="'CS-62'!A1" tooltip="Abrir CS-62" display="PERFIL DE OTRO USUARIO" xr:uid="{435D24CE-22C8-4DF9-B5E0-0A2AC1ED81B7}"/>
     <hyperlink ref="B66" location="'CS-63'!A1" tooltip="Abrir CS-63" display="PANTALLA DE VALORACIONES Y COMENTARIOS" xr:uid="{35FF9D6C-7966-4489-B1F7-CF06F7E93422}"/>
@@ -42595,4 +42595,14 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
+  <scriptId id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01GTZEWCAWIM7TFMIJC5EK6T67Q653ALHS:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9jZXUzNjUtbXkuc2hhcmVwb2ludC5jb20vOnU6L2cvcGVyc29uYWwvam9hcXVpbl9kZXZpY2VudGVhYmFkX3VzcF9jZXVfZXMvSVFBV1F6OHlzUWtYU0s5UDM0ZTdzQ3p5QWRTbTYxSVhqT1Q0SWpWUnFrYmtJbTg"/>
+</scriptIds>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{579C8B5B-9FA1-4985-ACF6-918C4CBEE006}"/>
 </file>
</xml_diff>